<commit_message>
Incorporate beta review feedback
</commit_message>
<xml_diff>
--- a/artifacts/beta-handoff/jeff-outreach-beta-tracker.xlsx
+++ b/artifacts/beta-handoff/jeff-outreach-beta-tracker.xlsx
@@ -41,11 +41,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,16 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -433,21 +438,21 @@
   <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="55" customWidth="1" min="14" max="14"/>
-    <col width="70" customWidth="1" min="15" max="15"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,7 +532,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="86" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>New Castle Building Products</t>
@@ -595,16 +600,16 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Jeff Paduto reviews/sends Maria warm-path draft or requests edits</t>
+          <t>Jeff Peduto reviews/sends Maria warm-path draft or requests edits</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Sender confirmed as Jeff Paduto. No attachment. Joe Boufard context approved. No known conflict confirmed.</t>
+          <t>Sender confirmed as Jeff Peduto. No attachment. Joe Bouffard context approved. No known conflict confirmed.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="86" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Colony Grill</t>
@@ -672,16 +677,16 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Jeff Paduto reviews/sends Ken warm-path draft or requests edits</t>
+          <t>Jeff Peduto reviews/sends Ken warm-path draft or requests edits</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Sender confirmed as Jeff Paduto. No attachment. Joe Boufard context approved. No known conflict confirmed.</t>
+          <t>Sender confirmed as Jeff Peduto. No attachment. Joe Bouffard context approved. No known conflict confirmed.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="86" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>TVG Fast and Fresh / Jimmy John's CT</t>
@@ -749,12 +754,12 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Jeff Paduto reviews/sends Will warm-path draft or requests edits</t>
+          <t>Jeff Peduto reviews/sends Will warm-path draft or requests edits</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Sender confirmed as Jeff Paduto. No attachment. Joe Boufard context approved. No known conflict confirmed. Lead with non-food operating categories due franchise constraints.</t>
+          <t>Sender confirmed as Jeff Peduto. No attachment. Joe Bouffard context approved. No known conflict confirmed. Lead with non-food operating categories due franchise constraints.</t>
         </is>
       </c>
     </row>

</xml_diff>